<commit_message>
Lots x2 joueurs par paire : lignes Joueur A / Joueur B distinctes
Chaque lot a 2 lignes (Joueur A + Joueur B) pour permettre
des lots différents au sein d'une même paire.
Total : 18 sélecteurs (4+3+2 lots x 2 joueurs).

https://claude.ai/code/session_01XUma5As6cQLzMdT7Bd3fVp
</commit_message>
<xml_diff>
--- a/budget_lots_padel.xlsx
+++ b/budget_lots_padel.xlsx
@@ -19,7 +19,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="#,##0.00 €"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="16">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -68,8 +68,26 @@
     </font>
     <font>
       <b val="1"/>
+      <color rgb="001A1A1A"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <color rgb="007BED5E"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <color rgb="00E8E8E8"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
     </font>
     <font>
       <b val="1"/>
@@ -198,7 +216,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -230,47 +248,59 @@
     <xf numFmtId="164" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="6" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="10" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="14" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="11" fillId="2" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="15" fillId="2" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -668,7 +698,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H30"/>
+  <dimension ref="A1:H50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -771,7 +801,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="22" customHeight="1">
+    <row r="7" ht="24" customHeight="1">
       <c r="A7" s="9" t="n">
         <v>1</v>
       </c>
@@ -787,16 +817,13 @@
       <c r="E7" s="1" t="n"/>
       <c r="F7" s="13" t="inlineStr">
         <is>
-          <t>1ER - Lot 1</t>
+          <t>1ER  (4 lots max)</t>
         </is>
       </c>
       <c r="G7" s="14" t="n"/>
-      <c r="H7" s="12">
-        <f>IF(G7="",0,VLOOKUP(G7,$B$7:$D$18,3,FALSE))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="8" ht="22" customHeight="1">
+      <c r="H7" s="14" t="n"/>
+    </row>
+    <row r="8" ht="20" customHeight="1">
       <c r="A8" s="15" t="n">
         <v>2</v>
       </c>
@@ -810,18 +837,18 @@
         <v>6</v>
       </c>
       <c r="E8" s="1" t="n"/>
-      <c r="F8" s="13" t="inlineStr">
-        <is>
-          <t>Lot 2</t>
-        </is>
-      </c>
-      <c r="G8" s="14" t="n"/>
+      <c r="F8" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Lot 1 - Joueur A</t>
+        </is>
+      </c>
+      <c r="G8" s="20" t="n"/>
       <c r="H8" s="12">
         <f>IF(G8="",0,VLOOKUP(G8,$B$7:$D$18,3,FALSE))</f>
         <v/>
       </c>
     </row>
-    <row r="9" ht="22" customHeight="1">
+    <row r="9" ht="20" customHeight="1">
       <c r="A9" s="9" t="n">
         <v>3</v>
       </c>
@@ -835,18 +862,18 @@
         <v>5</v>
       </c>
       <c r="E9" s="1" t="n"/>
-      <c r="F9" s="13" t="inlineStr">
-        <is>
-          <t>Lot 3</t>
-        </is>
-      </c>
-      <c r="G9" s="14" t="n"/>
-      <c r="H9" s="12">
+      <c r="F9" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">          Joueur B</t>
+        </is>
+      </c>
+      <c r="G9" s="22" t="n"/>
+      <c r="H9" s="18">
         <f>IF(G9="",0,VLOOKUP(G9,$B$7:$D$18,3,FALSE))</f>
         <v/>
       </c>
     </row>
-    <row r="10" ht="22" customHeight="1">
+    <row r="10" ht="20" customHeight="1">
       <c r="A10" s="15" t="n">
         <v>4</v>
       </c>
@@ -860,12 +887,12 @@
         <v>12</v>
       </c>
       <c r="E10" s="1" t="n"/>
-      <c r="F10" s="13" t="inlineStr">
-        <is>
-          <t>Lot 4</t>
-        </is>
-      </c>
-      <c r="G10" s="14" t="n"/>
+      <c r="F10" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Lot 2 - Joueur A</t>
+        </is>
+      </c>
+      <c r="G10" s="20" t="n"/>
       <c r="H10" s="12">
         <f>IF(G10="",0,VLOOKUP(G10,$B$7:$D$18,3,FALSE))</f>
         <v/>
@@ -885,18 +912,18 @@
         <v>10</v>
       </c>
       <c r="E11" s="1" t="n"/>
-      <c r="F11" s="19" t="inlineStr">
-        <is>
-          <t>S/Total 1ER</t>
-        </is>
-      </c>
-      <c r="G11" s="20" t="n"/>
-      <c r="H11" s="21">
-        <f>SUM(H7:H10)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="12" ht="22" customHeight="1">
+      <c r="F11" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">          Joueur B</t>
+        </is>
+      </c>
+      <c r="G11" s="22" t="n"/>
+      <c r="H11" s="18">
+        <f>IF(G11="",0,VLOOKUP(G11,$B$7:$D$18,3,FALSE))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12" ht="20" customHeight="1">
       <c r="A12" s="15" t="n">
         <v>6</v>
       </c>
@@ -910,18 +937,18 @@
         <v>9</v>
       </c>
       <c r="E12" s="1" t="n"/>
-      <c r="F12" s="22" t="inlineStr">
-        <is>
-          <t>2ÈME - Lot 1</t>
-        </is>
-      </c>
-      <c r="G12" s="14" t="n"/>
+      <c r="F12" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Lot 3 - Joueur A</t>
+        </is>
+      </c>
+      <c r="G12" s="20" t="n"/>
       <c r="H12" s="12">
         <f>IF(G12="",0,VLOOKUP(G12,$B$7:$D$18,3,FALSE))</f>
         <v/>
       </c>
     </row>
-    <row r="13" ht="22" customHeight="1">
+    <row r="13" ht="20" customHeight="1">
       <c r="A13" s="9" t="n">
         <v>7</v>
       </c>
@@ -935,18 +962,18 @@
         <v>15</v>
       </c>
       <c r="E13" s="1" t="n"/>
-      <c r="F13" s="22" t="inlineStr">
-        <is>
-          <t>Lot 2</t>
-        </is>
-      </c>
-      <c r="G13" s="14" t="n"/>
-      <c r="H13" s="12">
+      <c r="F13" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">          Joueur B</t>
+        </is>
+      </c>
+      <c r="G13" s="22" t="n"/>
+      <c r="H13" s="18">
         <f>IF(G13="",0,VLOOKUP(G13,$B$7:$D$18,3,FALSE))</f>
         <v/>
       </c>
     </row>
-    <row r="14" ht="22" customHeight="1">
+    <row r="14" ht="20" customHeight="1">
       <c r="A14" s="15" t="n">
         <v>8</v>
       </c>
@@ -960,12 +987,12 @@
         <v>18</v>
       </c>
       <c r="E14" s="1" t="n"/>
-      <c r="F14" s="22" t="inlineStr">
-        <is>
-          <t>Lot 3</t>
-        </is>
-      </c>
-      <c r="G14" s="14" t="n"/>
+      <c r="F14" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Lot 4 - Joueur A</t>
+        </is>
+      </c>
+      <c r="G14" s="20" t="n"/>
       <c r="H14" s="12">
         <f>IF(G14="",0,VLOOKUP(G14,$B$7:$D$18,3,FALSE))</f>
         <v/>
@@ -985,14 +1012,14 @@
         <v>16</v>
       </c>
       <c r="E15" s="1" t="n"/>
-      <c r="F15" s="19" t="inlineStr">
-        <is>
-          <t>S/Total 2ÈME</t>
-        </is>
-      </c>
-      <c r="G15" s="20" t="n"/>
-      <c r="H15" s="21">
-        <f>SUM(H12:H14)</f>
+      <c r="F15" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">          Joueur B</t>
+        </is>
+      </c>
+      <c r="G15" s="22" t="n"/>
+      <c r="H15" s="18">
+        <f>IF(G15="",0,VLOOKUP(G15,$B$7:$D$18,3,FALSE))</f>
         <v/>
       </c>
     </row>
@@ -1012,16 +1039,16 @@
       <c r="E16" s="1" t="n"/>
       <c r="F16" s="23" t="inlineStr">
         <is>
-          <t>3ÈME - Lot 1</t>
-        </is>
-      </c>
-      <c r="G16" s="14" t="n"/>
-      <c r="H16" s="12">
-        <f>IF(G16="",0,VLOOKUP(G16,$B$7:$D$18,3,FALSE))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17" ht="22" customHeight="1">
+          <t>S/Total 1ER</t>
+        </is>
+      </c>
+      <c r="G16" s="24" t="n"/>
+      <c r="H16" s="25">
+        <f>SUM(H8:H15)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17" ht="24" customHeight="1">
       <c r="A17" s="9" t="n">
         <v>11</v>
       </c>
@@ -1035,16 +1062,13 @@
         <v>25</v>
       </c>
       <c r="E17" s="1" t="n"/>
-      <c r="F17" s="23" t="inlineStr">
-        <is>
-          <t>Lot 2</t>
-        </is>
-      </c>
-      <c r="G17" s="14" t="n"/>
-      <c r="H17" s="12">
-        <f>IF(G17="",0,VLOOKUP(G17,$B$7:$D$18,3,FALSE))</f>
-        <v/>
-      </c>
+      <c r="F17" s="26" t="inlineStr">
+        <is>
+          <t>2ÈME  (3 lots max)</t>
+        </is>
+      </c>
+      <c r="G17" s="27" t="n"/>
+      <c r="H17" s="27" t="n"/>
     </row>
     <row r="18" ht="20" customHeight="1">
       <c r="A18" s="15" t="n">
@@ -1062,148 +1086,429 @@
       <c r="E18" s="1" t="n"/>
       <c r="F18" s="19" t="inlineStr">
         <is>
-          <t>S/Total 3ÈME</t>
+          <t xml:space="preserve">  Lot 1 - Joueur A</t>
         </is>
       </c>
       <c r="G18" s="20" t="n"/>
-      <c r="H18" s="21">
-        <f>SUM(H16:H17)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19" ht="4" customHeight="1">
+      <c r="H18" s="12">
+        <f>IF(G18="",0,VLOOKUP(G18,$B$7:$D$18,3,FALSE))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19" ht="20" customHeight="1">
       <c r="A19" s="1" t="n"/>
       <c r="B19" s="1" t="n"/>
       <c r="C19" s="1" t="n"/>
       <c r="D19" s="1" t="n"/>
       <c r="E19" s="1" t="n"/>
-      <c r="F19" s="6" t="n"/>
-      <c r="G19" s="6" t="n"/>
-      <c r="H19" s="6" t="n"/>
-    </row>
-    <row r="20" ht="30" customHeight="1">
+      <c r="F19" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">          Joueur B</t>
+        </is>
+      </c>
+      <c r="G19" s="22" t="n"/>
+      <c r="H19" s="18">
+        <f>IF(G19="",0,VLOOKUP(G19,$B$7:$D$18,3,FALSE))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20" ht="20" customHeight="1">
       <c r="A20" s="1" t="n"/>
       <c r="B20" s="1" t="n"/>
       <c r="C20" s="1" t="n"/>
       <c r="D20" s="1" t="n"/>
       <c r="E20" s="1" t="n"/>
-      <c r="F20" s="24" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="G20" s="25" t="n"/>
-      <c r="H20" s="26">
-        <f>H11+H15+H18</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21" ht="30" customHeight="1">
+      <c r="F20" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Lot 2 - Joueur A</t>
+        </is>
+      </c>
+      <c r="G20" s="20" t="n"/>
+      <c r="H20" s="12">
+        <f>IF(G20="",0,VLOOKUP(G20,$B$7:$D$18,3,FALSE))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21" ht="20" customHeight="1">
       <c r="A21" s="1" t="n"/>
       <c r="B21" s="1" t="n"/>
       <c r="C21" s="1" t="n"/>
       <c r="D21" s="1" t="n"/>
       <c r="E21" s="1" t="n"/>
-      <c r="F21" s="27" t="inlineStr">
-        <is>
-          <t>RESTE</t>
-        </is>
-      </c>
-      <c r="G21" s="28" t="n"/>
-      <c r="H21" s="29">
-        <f>84-H20</f>
-        <v/>
-      </c>
-    </row>
-    <row r="22">
+      <c r="F21" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">          Joueur B</t>
+        </is>
+      </c>
+      <c r="G21" s="22" t="n"/>
+      <c r="H21" s="18">
+        <f>IF(G21="",0,VLOOKUP(G21,$B$7:$D$18,3,FALSE))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22" ht="20" customHeight="1">
       <c r="A22" s="1" t="n"/>
       <c r="B22" s="1" t="n"/>
       <c r="C22" s="1" t="n"/>
       <c r="D22" s="1" t="n"/>
       <c r="E22" s="1" t="n"/>
-      <c r="F22" s="1" t="n"/>
-      <c r="G22" s="1" t="n"/>
-      <c r="H22" s="1" t="n"/>
-    </row>
-    <row r="23">
+      <c r="F22" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Lot 3 - Joueur A</t>
+        </is>
+      </c>
+      <c r="G22" s="20" t="n"/>
+      <c r="H22" s="12">
+        <f>IF(G22="",0,VLOOKUP(G22,$B$7:$D$18,3,FALSE))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23" ht="20" customHeight="1">
       <c r="A23" s="1" t="n"/>
       <c r="B23" s="1" t="n"/>
       <c r="C23" s="1" t="n"/>
       <c r="D23" s="1" t="n"/>
       <c r="E23" s="1" t="n"/>
-      <c r="F23" s="1" t="n"/>
-      <c r="G23" s="1" t="n"/>
-      <c r="H23" s="1" t="n"/>
-    </row>
-    <row r="24">
+      <c r="F23" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">          Joueur B</t>
+        </is>
+      </c>
+      <c r="G23" s="22" t="n"/>
+      <c r="H23" s="18">
+        <f>IF(G23="",0,VLOOKUP(G23,$B$7:$D$18,3,FALSE))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24" ht="22" customHeight="1">
       <c r="A24" s="1" t="n"/>
       <c r="B24" s="1" t="n"/>
       <c r="C24" s="1" t="n"/>
       <c r="D24" s="1" t="n"/>
       <c r="E24" s="1" t="n"/>
-      <c r="F24" s="1" t="n"/>
-      <c r="G24" s="1" t="n"/>
-      <c r="H24" s="1" t="n"/>
-    </row>
-    <row r="25">
+      <c r="F24" s="23" t="inlineStr">
+        <is>
+          <t>S/Total 2ÈME</t>
+        </is>
+      </c>
+      <c r="G24" s="24" t="n"/>
+      <c r="H24" s="25">
+        <f>SUM(H18:H23)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25" ht="24" customHeight="1">
       <c r="A25" s="1" t="n"/>
       <c r="B25" s="1" t="n"/>
       <c r="C25" s="1" t="n"/>
       <c r="D25" s="1" t="n"/>
       <c r="E25" s="1" t="n"/>
-      <c r="F25" s="1" t="n"/>
-      <c r="G25" s="1" t="n"/>
-      <c r="H25" s="1" t="n"/>
-    </row>
-    <row r="26">
+      <c r="F25" s="28" t="inlineStr">
+        <is>
+          <t>3ÈME  (2 lots max)</t>
+        </is>
+      </c>
+      <c r="G25" s="29" t="n"/>
+      <c r="H25" s="29" t="n"/>
+    </row>
+    <row r="26" ht="20" customHeight="1">
       <c r="A26" s="1" t="n"/>
       <c r="B26" s="1" t="n"/>
       <c r="C26" s="1" t="n"/>
       <c r="D26" s="1" t="n"/>
       <c r="E26" s="1" t="n"/>
-      <c r="F26" s="1" t="n"/>
-      <c r="G26" s="1" t="n"/>
-      <c r="H26" s="1" t="n"/>
-    </row>
-    <row r="27">
+      <c r="F26" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Lot 1 - Joueur A</t>
+        </is>
+      </c>
+      <c r="G26" s="20" t="n"/>
+      <c r="H26" s="12">
+        <f>IF(G26="",0,VLOOKUP(G26,$B$7:$D$18,3,FALSE))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27" ht="20" customHeight="1">
       <c r="A27" s="1" t="n"/>
       <c r="B27" s="1" t="n"/>
       <c r="C27" s="1" t="n"/>
       <c r="D27" s="1" t="n"/>
       <c r="E27" s="1" t="n"/>
-      <c r="F27" s="1" t="n"/>
-      <c r="G27" s="1" t="n"/>
-      <c r="H27" s="1" t="n"/>
-    </row>
-    <row r="28">
+      <c r="F27" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">          Joueur B</t>
+        </is>
+      </c>
+      <c r="G27" s="22" t="n"/>
+      <c r="H27" s="18">
+        <f>IF(G27="",0,VLOOKUP(G27,$B$7:$D$18,3,FALSE))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28" ht="20" customHeight="1">
       <c r="A28" s="1" t="n"/>
       <c r="B28" s="1" t="n"/>
       <c r="C28" s="1" t="n"/>
       <c r="D28" s="1" t="n"/>
       <c r="E28" s="1" t="n"/>
-      <c r="F28" s="1" t="n"/>
-      <c r="G28" s="1" t="n"/>
-      <c r="H28" s="1" t="n"/>
-    </row>
-    <row r="29">
+      <c r="F28" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Lot 2 - Joueur A</t>
+        </is>
+      </c>
+      <c r="G28" s="20" t="n"/>
+      <c r="H28" s="12">
+        <f>IF(G28="",0,VLOOKUP(G28,$B$7:$D$18,3,FALSE))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29" ht="20" customHeight="1">
       <c r="A29" s="1" t="n"/>
       <c r="B29" s="1" t="n"/>
       <c r="C29" s="1" t="n"/>
       <c r="D29" s="1" t="n"/>
       <c r="E29" s="1" t="n"/>
-      <c r="F29" s="1" t="n"/>
-      <c r="G29" s="1" t="n"/>
-      <c r="H29" s="1" t="n"/>
-    </row>
-    <row r="30">
+      <c r="F29" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">          Joueur B</t>
+        </is>
+      </c>
+      <c r="G29" s="22" t="n"/>
+      <c r="H29" s="18">
+        <f>IF(G29="",0,VLOOKUP(G29,$B$7:$D$18,3,FALSE))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30" ht="22" customHeight="1">
       <c r="A30" s="1" t="n"/>
       <c r="B30" s="1" t="n"/>
       <c r="C30" s="1" t="n"/>
       <c r="D30" s="1" t="n"/>
       <c r="E30" s="1" t="n"/>
-      <c r="F30" s="1" t="n"/>
-      <c r="G30" s="1" t="n"/>
-      <c r="H30" s="1" t="n"/>
+      <c r="F30" s="23" t="inlineStr">
+        <is>
+          <t>S/Total 3ÈME</t>
+        </is>
+      </c>
+      <c r="G30" s="24" t="n"/>
+      <c r="H30" s="25">
+        <f>SUM(H26:H29)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31" ht="4" customHeight="1">
+      <c r="A31" s="1" t="n"/>
+      <c r="B31" s="1" t="n"/>
+      <c r="C31" s="1" t="n"/>
+      <c r="D31" s="1" t="n"/>
+      <c r="E31" s="1" t="n"/>
+      <c r="F31" s="6" t="n"/>
+      <c r="G31" s="6" t="n"/>
+      <c r="H31" s="6" t="n"/>
+    </row>
+    <row r="32" ht="30" customHeight="1">
+      <c r="A32" s="1" t="n"/>
+      <c r="B32" s="1" t="n"/>
+      <c r="C32" s="1" t="n"/>
+      <c r="D32" s="1" t="n"/>
+      <c r="E32" s="1" t="n"/>
+      <c r="F32" s="30" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="G32" s="31" t="n"/>
+      <c r="H32" s="32">
+        <f>H16+H24+H30</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33" ht="30" customHeight="1">
+      <c r="A33" s="1" t="n"/>
+      <c r="B33" s="1" t="n"/>
+      <c r="C33" s="1" t="n"/>
+      <c r="D33" s="1" t="n"/>
+      <c r="E33" s="1" t="n"/>
+      <c r="F33" s="33" t="inlineStr">
+        <is>
+          <t>RESTE</t>
+        </is>
+      </c>
+      <c r="G33" s="34" t="n"/>
+      <c r="H33" s="35">
+        <f>84-H32</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="1" t="n"/>
+      <c r="B34" s="1" t="n"/>
+      <c r="C34" s="1" t="n"/>
+      <c r="D34" s="1" t="n"/>
+      <c r="E34" s="1" t="n"/>
+      <c r="F34" s="1" t="n"/>
+      <c r="G34" s="1" t="n"/>
+      <c r="H34" s="1" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="1" t="n"/>
+      <c r="B35" s="1" t="n"/>
+      <c r="C35" s="1" t="n"/>
+      <c r="D35" s="1" t="n"/>
+      <c r="E35" s="1" t="n"/>
+      <c r="F35" s="1" t="n"/>
+      <c r="G35" s="1" t="n"/>
+      <c r="H35" s="1" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="1" t="n"/>
+      <c r="B36" s="1" t="n"/>
+      <c r="C36" s="1" t="n"/>
+      <c r="D36" s="1" t="n"/>
+      <c r="E36" s="1" t="n"/>
+      <c r="F36" s="1" t="n"/>
+      <c r="G36" s="1" t="n"/>
+      <c r="H36" s="1" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="1" t="n"/>
+      <c r="B37" s="1" t="n"/>
+      <c r="C37" s="1" t="n"/>
+      <c r="D37" s="1" t="n"/>
+      <c r="E37" s="1" t="n"/>
+      <c r="F37" s="1" t="n"/>
+      <c r="G37" s="1" t="n"/>
+      <c r="H37" s="1" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="1" t="n"/>
+      <c r="B38" s="1" t="n"/>
+      <c r="C38" s="1" t="n"/>
+      <c r="D38" s="1" t="n"/>
+      <c r="E38" s="1" t="n"/>
+      <c r="F38" s="1" t="n"/>
+      <c r="G38" s="1" t="n"/>
+      <c r="H38" s="1" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="1" t="n"/>
+      <c r="B39" s="1" t="n"/>
+      <c r="C39" s="1" t="n"/>
+      <c r="D39" s="1" t="n"/>
+      <c r="E39" s="1" t="n"/>
+      <c r="F39" s="1" t="n"/>
+      <c r="G39" s="1" t="n"/>
+      <c r="H39" s="1" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="1" t="n"/>
+      <c r="B40" s="1" t="n"/>
+      <c r="C40" s="1" t="n"/>
+      <c r="D40" s="1" t="n"/>
+      <c r="E40" s="1" t="n"/>
+      <c r="F40" s="1" t="n"/>
+      <c r="G40" s="1" t="n"/>
+      <c r="H40" s="1" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="1" t="n"/>
+      <c r="B41" s="1" t="n"/>
+      <c r="C41" s="1" t="n"/>
+      <c r="D41" s="1" t="n"/>
+      <c r="E41" s="1" t="n"/>
+      <c r="F41" s="1" t="n"/>
+      <c r="G41" s="1" t="n"/>
+      <c r="H41" s="1" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="1" t="n"/>
+      <c r="B42" s="1" t="n"/>
+      <c r="C42" s="1" t="n"/>
+      <c r="D42" s="1" t="n"/>
+      <c r="E42" s="1" t="n"/>
+      <c r="F42" s="1" t="n"/>
+      <c r="G42" s="1" t="n"/>
+      <c r="H42" s="1" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="1" t="n"/>
+      <c r="B43" s="1" t="n"/>
+      <c r="C43" s="1" t="n"/>
+      <c r="D43" s="1" t="n"/>
+      <c r="E43" s="1" t="n"/>
+      <c r="F43" s="1" t="n"/>
+      <c r="G43" s="1" t="n"/>
+      <c r="H43" s="1" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="1" t="n"/>
+      <c r="B44" s="1" t="n"/>
+      <c r="C44" s="1" t="n"/>
+      <c r="D44" s="1" t="n"/>
+      <c r="E44" s="1" t="n"/>
+      <c r="F44" s="1" t="n"/>
+      <c r="G44" s="1" t="n"/>
+      <c r="H44" s="1" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="1" t="n"/>
+      <c r="B45" s="1" t="n"/>
+      <c r="C45" s="1" t="n"/>
+      <c r="D45" s="1" t="n"/>
+      <c r="E45" s="1" t="n"/>
+      <c r="F45" s="1" t="n"/>
+      <c r="G45" s="1" t="n"/>
+      <c r="H45" s="1" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="1" t="n"/>
+      <c r="B46" s="1" t="n"/>
+      <c r="C46" s="1" t="n"/>
+      <c r="D46" s="1" t="n"/>
+      <c r="E46" s="1" t="n"/>
+      <c r="F46" s="1" t="n"/>
+      <c r="G46" s="1" t="n"/>
+      <c r="H46" s="1" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="1" t="n"/>
+      <c r="B47" s="1" t="n"/>
+      <c r="C47" s="1" t="n"/>
+      <c r="D47" s="1" t="n"/>
+      <c r="E47" s="1" t="n"/>
+      <c r="F47" s="1" t="n"/>
+      <c r="G47" s="1" t="n"/>
+      <c r="H47" s="1" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="1" t="n"/>
+      <c r="B48" s="1" t="n"/>
+      <c r="C48" s="1" t="n"/>
+      <c r="D48" s="1" t="n"/>
+      <c r="E48" s="1" t="n"/>
+      <c r="F48" s="1" t="n"/>
+      <c r="G48" s="1" t="n"/>
+      <c r="H48" s="1" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="1" t="n"/>
+      <c r="B49" s="1" t="n"/>
+      <c r="C49" s="1" t="n"/>
+      <c r="D49" s="1" t="n"/>
+      <c r="E49" s="1" t="n"/>
+      <c r="F49" s="1" t="n"/>
+      <c r="G49" s="1" t="n"/>
+      <c r="H49" s="1" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="1" t="n"/>
+      <c r="B50" s="1" t="n"/>
+      <c r="C50" s="1" t="n"/>
+      <c r="D50" s="1" t="n"/>
+      <c r="E50" s="1" t="n"/>
+      <c r="F50" s="1" t="n"/>
+      <c r="G50" s="1" t="n"/>
+      <c r="H50" s="1" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -1213,7 +1518,7 @@
     <mergeCell ref="C4:D4"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="G7 G8 G9 G10 G12 G13 G14 G16 G17" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Lot invalide" error="Choisissez un lot du catalogue" promptTitle="Choix du lot" prompt="Sélectionnez un lot du catalogue" type="list">
+    <dataValidation sqref="G8 G9 G10 G11 G12 G13 G14 G15 G18 G19 G20 G21 G22 G23 G26 G27 G28 G29" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Lot invalide" error="Choisissez un lot du catalogue" promptTitle="Choix du lot" prompt="Sélectionnez un lot du catalogue" type="list">
       <formula1>=$B$7:$B$18</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>